<commit_message>
feat(F-NAR-008): 16 ATOM de plus + voix plus lentes
Vague COR/NOM appliquée. Brief : vraie histoire (monde, imprévu, fin vécue),
plus de « L'histoire est finie ». Piper : pitch enfant baissé, silences plus longs.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-07.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-07.xlsx
@@ -2117,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2188,6 +2188,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-07 Le carton-tunnel d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-07.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chemin du parc après la pluie</t>
+          <t>chemin du parc après la pluie, terre, fil d'argent, limace</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aniss, Chouchou, papa</t>
+          <t>Aniss, Chouchou, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut faire passer le ballon jaune dans un carton-tunnel. Le carton ramollit. Chouchou tient les bords. Le ballon sort de l'autre côté.</t>
+          <t>Une odeur de champignon monte du chemin. Sur le fil d'argent, un éclat de limace brille. Aniss veut un tunnel pour le ballon jaune, maintenant. Il pousse trop vite : le carton mouillé s'écrase. Chouchou veut la limace. Un rire commence, puis s'arrête. Il refuse de foncer. Ils tiennent les bords. Merci vécu. Il se glisse trop vite : ça colle. Il refuse, retrouve l'éclat. Un éclat de limace tient sur le fil.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La terre du chemin sent le champignon. Un fil d'argent brille sur la pierre. C'est une limace, toute lente. Le banc a encore une tache d'eau. Papa pose un carton sur l'herbe. Le carton sent le papier humide. Tu as vu le fil d'argent, Aniss ? Il brille. Oui. La limace va tout doux. En ce moment, Aniss touche le ballon jaune. Le caoutchouc est froid et lisse. Je veux un tunnel. Avec le carton. Le ballon passe dedans ? Oui. Et il sort de l'autre côté. Aniss pousse le carton près du banc. L'herbe mouille ses genoux. Ça sent le vert et la terre. Chouchou arrive près du chemin. Ses bottes font un bruit mou. Chouchou est plus rond. Aniss est plus mince. On joue ensemble. Le corps n'est pas une blague. Tu tiens le carton, Chouchou ? Oui. Chouchou tient un bord. Aniss tient l'autre bord. Le carton tremble un peu. Il est mou. La pluie l'a mouillé. Aniss pousse le ballon. Le ballon entre dans le carton. Le carton s'écrase tout doux. Oh. Il reste coincé. On peut le tenir plus fort. Ensemble.</t>
+          <t>Une odeur de champignon monte du chemin. Ça sent la terre, papa ! Tu le sens, après la pluie ? Oui, un peu froid. Un fil d'argent brille sur la pierre. Il brille, maman. C'est la limace, sur la pierre ? Oui, un petit fil. La limace avance, très lente. Sur le fil, un éclat de limace brille. Il est petit, papa. C'est l'eau, sous la lumière. Oui, un petit point. Le banc garde une tache d'eau. Elle est froide. On reste près du banc ? Oui, maman. Papa pose un carton sur l'herbe. Le carton sent le papier humide. Il est mou. La pluie l'a mouillé, Aniss ? Oui, papa. Maman pose le ballon jaune près du carton. Le caoutchouc est froid, Aniss. Il est lisse. Je veux un tunnel, maintenant ! Avec le carton, sur l'herbe ? Oui. Le ballon passe dedans. Et il sort de l'autre côté ? Oui, maman. Chouchou arrive près du chemin. Ses bottes font un bruit mou. Chouchou ! J'arrive. Le tunnel, maintenant, Chouchou ! En ce moment, Aniss pousse le carton trop vite. L'herbe mouille ses genoux. Le carton s'écrase, tout plat. Oh. Tu tiens le bord, tout de suite ! Aniss attrape la manche de Chouchou. Non. Chouchou recule vers la pierre. Elle regarde la limace, longtemps. Oh. Le carton mouillé reste sur le dos de Chouchou. Il est drôle, sur toi ! Un rire commence dans la bouche d'Aniss. Chouchou ne dit rien. Le sourire de Chouchou disparaît. Pousse, maintenant ! Non. Oh. Aniss pousse le ballon tout seul. Le ballon reste coincé, sous le papier. Il reste coincé ! Oh. L'éclat de limace tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Le carton est plat, Aniss ? Papa s'accroupit à la même hauteur. Oui, papa. Chouchou est près de la pierre, Aniss. Oui, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La terre du chemin sent le champignon. Un fil d'argent brille sur la pierre. C'est une limace, toute lente. Le banc a encore une tache d'eau. Papa pose un carton sur l'herbe. Le carton sent le papier humide. Tu as vu le fil d'argent, Aniss ? Il brille. Oui. La limace va tout doux. En ce moment, Aniss touche le ballon jaune. Le caoutchouc est froid et lisse. Je veux un tunnel. Avec le carton. Le ballon passe dedans ? Oui. Et il sort de l'autre côté. Aniss pousse le carton près du banc. L'herbe mouille ses genoux. Ça sent le vert et la terre. Chouchou arrive près du chemin. Ses bottes font un bruit mou. Chouchou est plus rond. Aniss est plus mince. On joue ensemble. Le corps n'est pas une blague. Tu tiens le carton, Chouchou ? Oui. Chouchou tient un bord. Aniss tient l'autre bord. Le carton tremble un peu. Il est mou. La pluie l'a mouillé. Aniss pousse le ballon. Le ballon entre dans le carton. Le carton s'écrase tout doux. Oh. Il reste coincé. On peut le tenir plus fort. Ensemble.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une odeur de champignon monte du chemin. Ça sent la terre, papa ! Tu le sens, après la pluie ? Oui, un peu froid. Un fil d'argent brille sur la pierre. Il brille, maman. C'est la limace, sur la pierre ? Oui, un petit fil. La limace avance, très lente. Sur le fil, un &lt;emphasis level="moderate"&gt;éclat de limace&lt;/emphasis&gt; brille. Il est petit, papa. C'est l'eau, sous la lumière. Oui, un petit point. Le banc garde une tache d'eau. Elle est froide. On reste près du banc ? Oui, maman. Papa pose un carton sur l'herbe. Le carton sent le papier humide. Il est mou. La pluie l'a mouillé, Aniss ? Oui, papa. Maman pose le ballon jaune près du carton. Le caoutchouc est froid, Aniss. Il est lisse. Je veux un tunnel, maintenant ! Avec le carton, sur l'herbe ? Oui. Le ballon passe dedans. Et il sort de l'autre côté ? Oui, maman. Chouchou arrive près du chemin. Ses bottes font un bruit mou. Chouchou ! J'arrive. Le tunnel, maintenant, Chouchou ! En ce moment, Aniss pousse le carton trop vite. L'herbe mouille ses genoux. Le carton s'écrase, tout plat. Oh. Tu tiens le bord, tout de suite ! Aniss attrape la manche de Chouchou. Non. Chouchou recule vers la pierre. Elle regarde la limace, longtemps. Oh. Le carton mouillé reste sur le dos de Chouchou. Il est drôle, sur toi ! Un rire commence dans la bouche d'Aniss. Chouchou ne dit rien. Le sourire de Chouchou disparaît. Pousse, maintenant ! Non. Oh. Aniss pousse le ballon tout seul. Le ballon reste coincé, sous le papier. Il reste coincé ! Oh. L'éclat de limace tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Le carton est plat, Aniss ? Papa s'accroupit à la même hauteur. Oui, papa. Chouchou est près de la pierre, Aniss. Oui, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Delphine et Erwan sont au parc avec papa. Ils se passent un ballon. Erwan a un &lt;emphasis&gt;corps&lt;/emphasis&gt; plus rond. Delphine a un corps plus mince. Papa dit : le corps n'est pas une blague. On joue ensemble. Delphine ne commente pas le corps. Elle passe le ballon. Erwan le rend. Ils rient du jeu, pas du corps. L'amitié ne dépend pas de la forme. On joue. Le corps n'est pas une blague. [pause]</t>
+          <t>Une odeur de champignon monte du chemin. Ça sent la terre, papa ! Tu le sens, après la pluie ? Oui, un peu froid. Un fil d'argent brille sur la pierre. Il brille, maman. C'est la limace, sur la pierre ? Oui, un petit fil. La limace avance, très lente. Sur le fil, un &lt;emphasis&gt;éclat de limace&lt;/emphasis&gt; brille. Il est petit, papa. C'est l'eau, sous la lumière. Oui, un petit point. Le banc garde une tache d'eau. Elle est froide. On reste près du banc ? Oui, maman. Papa pose un carton sur l'herbe. Le carton sent le papier humide. Il est mou. La pluie l'a mouillé, Aniss ? Oui, papa. Maman pose le ballon jaune près du carton. Le caoutchouc est froid, Aniss. Il est lisse. Je veux un tunnel, maintenant ! Avec le carton, sur l'herbe ? Oui. Le ballon passe dedans. Et il sort de l'autre côté ? Oui, maman. Chouchou arrive près du chemin. Ses bottes font un bruit mou. Chouchou ! J'arrive. Le tunnel, maintenant, Chouchou ! En ce moment, Aniss pousse le carton trop vite. L'herbe mouille ses genoux. Le carton s'écrase, tout plat. Oh. Tu tiens le bord, tout de suite ! Aniss attrape la manche de Chouchou. Non. Chouchou recule vers la pierre. Elle regarde la limace, longtemps. Oh. Le carton mouillé reste sur le dos de Chouchou. Il est drôle, sur toi ! Un rire commence dans la bouche d'Aniss. Chouchou ne dit rien. Le sourire de Chouchou disparaît. Pousse, maintenant ! Non. Oh. Aniss pousse le ballon tout seul. Le ballon reste coincé, sous le papier. Il reste coincé ! Oh. L'éclat de limace tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Le carton est plat, Aniss ? Papa s'accroupit à la même hauteur. Oui, papa. Chouchou est près de la pierre, Aniss. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de limace</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,49 +1321,80 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_tunnel_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La terre du chemin sent le champignon.
+          <t>narrateur|Une odeur de champignon monte du chemin.
+enfant-m|Ça sent la terre, papa !
+papa|Tu le sens, après la pluie ?
+enfant-m|Oui, un peu froid.
 narrateur|Un fil d'argent brille sur la pierre.
-narrateur|C'est une limace, toute lente.
-narrateur|Le banc a encore une tache d'eau.
+enfant-m|Il brille, maman.
+maman|C'est la limace, sur la pierre ?
+enfant-m|Oui, un petit fil.
+narrateur|La limace avance, très lente.
+narrateur|Sur le fil, un éclat de limace brille.
+enfant-m|Il est petit, papa.
+papa|C'est l'eau, sous la lumière.
+enfant-m|Oui, un petit point.
+narrateur|Le banc garde une tache d'eau.
+enfant-m|Elle est froide.
+maman|On reste près du banc ?
+enfant-m|Oui, maman.
 narrateur|Papa pose un carton sur l'herbe.
 narrateur|Le carton sent le papier humide.
-papa|Tu as vu le fil d'argent, Aniss ?
-enfant-m|Il brille.
-papa|Oui.
-papa|La limace va tout doux.
-narrateur|En ce moment, Aniss touche le ballon jaune.
-narrateur|Le caoutchouc est froid et lisse.
-enfant-m|Je veux un tunnel.
-enfant-m|Avec le carton.
-papa|Le ballon passe dedans ?
+enfant-m|Il est mou.
+papa|La pluie l'a mouillé, Aniss ?
+enfant-m|Oui, papa.
+narrateur|Maman pose le ballon jaune près du carton.
+maman|Le caoutchouc est froid, Aniss.
+enfant-m|Il est lisse.
+enfant-m|Je veux un tunnel, maintenant !
+papa|Avec le carton, sur l'herbe ?
 enfant-m|Oui.
-papa|Et il sort de l'autre côté.
-narrateur|Aniss pousse le carton près du banc.
-narrateur|L'herbe mouille ses genoux.
-narrateur|Ça sent le vert et la terre.
+enfant-m|Le ballon passe dedans.
+maman|Et il sort de l'autre côté ?
+enfant-m|Oui, maman.
 narrateur|Chouchou arrive près du chemin.
 narrateur|Ses bottes font un bruit mou.
-narrateur|Chouchou est plus rond.
-narrateur|Aniss est plus mince.
-papa|On joue ensemble.
-papa|Le corps n'est pas une blague.
-enfant-m|Tu tiens le carton, Chouchou ?
-copain|Oui.
-narrateur|Chouchou tient un bord.
-narrateur|Aniss tient l'autre bord.
-narrateur|Le carton tremble un peu.
-enfant-m|Il est mou.
-papa|La pluie l'a mouillé.
-narrateur|Aniss pousse le ballon.
-narrateur|Le ballon entre dans le carton.
-narrateur|Le carton s'écrase tout doux.
+enfant-m|Chouchou !
+enfant-f|J'arrive.
+enfant-m|Le tunnel, maintenant, Chouchou !
+narrateur|En ce moment, Aniss pousse le carton trop vite.
+narrateur|L'herbe mouille ses genoux.
+narrateur|Le carton s'écrase, tout plat.
 enfant-m|Oh.
-copain|Il reste coincé.
-papa|On peut le tenir plus fort.
-papa|Ensemble.</t>
+enfant-m|Tu tiens le bord, tout de suite !
+narrateur|Aniss attrape la manche de Chouchou.
+enfant-f|Non.
+narrateur|Chouchou recule vers la pierre.
+narrateur|Elle regarde la limace, longtemps.
+enfant-m|Oh.
+narrateur|Le carton mouillé reste sur le dos de Chouchou.
+enfant-m|Il est drôle, sur toi !
+narrateur|Un rire commence dans la bouche d'Aniss.
+narrateur|Chouchou ne dit rien.
+narrateur|Le sourire de Chouchou disparaît.
+enfant-m|Pousse, maintenant !
+enfant-f|Non.
+enfant-m|Oh.
+narrateur|Aniss pousse le ballon tout seul.
+narrateur|Le ballon reste coincé, sous le papier.
+enfant-m|Il reste coincé !
+enfant-f|Oh.
+narrateur|L'éclat de limace tremble, puis tient.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+papa|Le carton est plat, Aniss ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-m|Oui, papa.
+maman|Chouchou est près de la pierre, Aniss.
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1400,12 +1431,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le carton s'écrase. Que font Aniss et Chouchou ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;carton&lt;/emphasis&gt; s'écrase. Que font Aniss et Chouchou ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Delphine joue avec Erwan. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;carton&lt;/emphasis&gt; s'écrase. Que font Aniss et Chouchou ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1468,7 +1499,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1476,10 +1507,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1525,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>carton</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,23 +1565,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=ils_tiennent_le_carton_ils_jouent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1579,17 +1614,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss appelle Chouchou. Ils tiennent le carton à deux. Vous tenez bien les bords. Merci, Aniss. Merci, Chouchou. Le carton redevient un tunnel. Pousse, Chouchou. J'aide. Aniss pousse le ballon tout doux. Le caoutchouc glisse sur le carton. Ça fait un bruit de papier. On joue ensemble. Le corps n'est pas une blague. Il va sortir ? Encore un peu.</t>
+          <t>Aniss veut le tunnel, tout de suite. Tu tiens, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près de la pierre. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il lâche la manche, un peu. Le carton est plat, Aniss ? Papa reste à sa hauteur. La limace avance, près de la pierre. Aniss attend que le silence arrive. On joue, Chouchou ? Tu tiens le bord, si tu veux ? Chouchou ne dit rien. Elle regarde le carton, longtemps. Je regarde. D'accord. Aniss redresse un bord du carton. L'autre bord reste dans l'herbe. Je tiens. Chouchou tient le bord, sans presser. Aniss pousse le ballon, plus léger. Le caoutchouc glisse sur le papier. Il entre ! Merci, Aniss. Papa a vu les deux, près du carton. Tes genoux sont mouillés, Aniss ? Un peu, maman. Le ballon est dedans. Tu as entendu le papier ? Oui, papa. On reste près du banc, Aniss ? Oui. Le ventre d'Aniss se desserre. Il va sortir ? Un peu, Aniss.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss appelle Chouchou. Ils tiennent le carton à deux. Vous tenez bien les bords. Merci, Aniss. Merci, Chouchou. Le carton redevient un tunnel. Pousse, Chouchou. J'aide. Aniss pousse le ballon tout doux. Le caoutchouc glisse sur le carton. Ça fait un bruit de papier. On joue ensemble. Le corps n'est pas une blague. Il va sortir ? Encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut le tunnel, tout de suite. Tu tiens, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près de la pierre. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il lâche la manche, un peu. Le carton est plat, Aniss ? Papa reste à sa hauteur. La limace avance, près de la pierre. Aniss attend que le silence arrive. &lt;emphasis level="moderate"&gt;On joue&lt;/emphasis&gt;, Chouchou ? Tu tiens le bord, si tu veux ? Chouchou ne dit rien. Elle regarde le carton, longtemps. Je regarde. D'accord. Aniss redresse un bord du carton. L'autre bord reste dans l'herbe. Je tiens. Chouchou tient le bord, sans presser. Aniss pousse le ballon, plus léger. Le caoutchouc glisse sur le papier. Il entre ! Merci, Aniss. Papa a vu les deux, près du carton. Tes genoux sont mouillés, Aniss ? Un peu, maman. Le ballon est dedans. Tu as entendu le papier ? Oui, papa. On reste près du banc, Aniss ? Oui. Le ventre d'Aniss se desserre. Il va sortir ? Un peu, Aniss.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Delphine a joué avec Erwan. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'était pas une blague. [pause]</t>
+          <t>Aniss veut le tunnel, tout de suite. Tu tiens, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près de la pierre. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il lâche la manche, un peu. Le carton est plat, Aniss ? Papa reste à sa hauteur. La limace avance, près de la pierre. Aniss attend que le silence arrive. &lt;emphasis&gt;On joue&lt;/emphasis&gt;, Chouchou ? Tu tiens le bord, si tu veux ? Chouchou ne dit rien. Elle regarde le carton, longtemps. Je regarde. D'accord. Aniss redresse un bord du carton. L'autre bord reste dans l'herbe. Je tiens. Chouchou tient le bord, sans presser. Aniss pousse le ballon, plus léger. Le caoutchouc glisse sur le papier. Il entre ! Merci, Aniss. Papa a vu les deux, près du carton. Tes genoux sont mouillés, Aniss ? Un peu, maman. Le ballon est dedans. Tu as entendu le papier ? Oui, papa. On reste près du banc, Aniss ? Oui. Le ventre d'Aniss se desserre. Il va sortir ? Un peu, Aniss. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1671,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1679,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1705,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>On joue</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1737,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,26 +1753,54 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_les_bords_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss appelle Chouchou.
-narrateur|Ils tiennent le carton à deux.
-papa|Vous tenez bien les bords.
+          <t>narrateur|Aniss veut le tunnel, tout de suite.
+enfant-m|Tu tiens, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Non.
+narrateur|Chouchou reste près de la pierre.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Aniss refuse de foncer.
+narrateur|Il lâche la manche, un peu.
+papa|Le carton est plat, Aniss ?
+narrateur|Papa reste à sa hauteur.
+maman|La limace avance, près de la pierre.
+narrateur|Aniss attend que le silence arrive.
+enfant-m|On joue, Chouchou ?
+enfant-m|Tu tiens le bord, si tu veux ?
+narrateur|Chouchou ne dit rien.
+narrateur|Elle regarde le carton, longtemps.
+enfant-f|Je regarde.
+enfant-m|D'accord.
+narrateur|Aniss redresse un bord du carton.
+narrateur|L'autre bord reste dans l'herbe.
+enfant-f|Je tiens.
+narrateur|Chouchou tient le bord, sans presser.
+narrateur|Aniss pousse le ballon, plus léger.
+narrateur|Le caoutchouc glisse sur le papier.
+enfant-m|Il entre !
 papa|Merci, Aniss.
-papa|Merci, Chouchou.
-narrateur|Le carton redevient un tunnel.
-enfant-m|Pousse, Chouchou.
-copain|J'aide.
-narrateur|Aniss pousse le ballon tout doux.
-narrateur|Le caoutchouc glisse sur le carton.
-narrateur|Ça fait un bruit de papier.
-papa|On joue ensemble.
-papa|Le corps n'est pas une blague.
+narrateur|Papa a vu les deux, près du carton.
+maman|Tes genoux sont mouillés, Aniss ?
+enfant-m|Un peu, maman.
+enfant-f|Le ballon est dedans.
+papa|Tu as entendu le papier ?
+enfant-m|Oui, papa.
+maman|On reste près du banc, Aniss ?
+enfant-m|Oui.
+narrateur|Le ventre d'Aniss se desserre.
 enfant-m|Il va sortir ?
-papa|Encore un peu.</t>
+maman|Un peu, Aniss.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>ballon,carton</t>
         </is>
       </c>
     </row>
@@ -1764,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le ballon sort de l'autre côté. Il fait poum dans l'herbe. Il est passé ! Poum. Bravo. Vous avez tenu le carton. Une goutte tombe du banc. Elle fait un rond dans l'eau. On le refait ? Encore. Chouchou redresse le bord. Aniss attend de l'autre côté. Le ballon traverse encore. Le carton tremble, puis tient. Poum. Le tunnel marche. Oui. Vous l'avez fait à deux. La limace a avancé d'un doigt. Le fil d'argent brille encore.</t>
+          <t>Aniss veut passer dans le tunnel. Moi, maintenant ! Il se glisse trop vite sous le carton. Le carton mouillé colle à son dos. Oh. Il reste collé. Un rire revient dans la bouche d'Aniss. Chouchou ne rit pas. Attends. Chouchou lâche le bord. Le carton s'écrase, une fois. Ça tombe ! Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le carton, un instant. Il écoute l'herbe, près du fil. Sur le fil, un éclat de limace luit. Il est là. On tient, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Ils tiennent les deux bords, à deux. Aniss pousse le ballon, plus lent. Le ballon sort de l'autre côté. Il fait poum dans l'herbe. Il est passé ! Poum. Tu restes un peu ? Oui, papa. Le carton est près du banc. On le laisse ? Oui, contre le bois. Une goutte tombe du banc. Elle fait un rond dans l'eau. Un rond, maman. Oui, dans l'eau.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le ballon sort de l'autre côté. Il fait poum dans l'herbe. Il est passé ! Poum. Bravo. Vous avez tenu le carton. Une goutte tombe du banc. Elle fait un rond dans l'eau. On le refait ? Encore. Chouchou redresse le bord. Aniss attend de l'autre côté. Le ballon traverse encore. Le carton tremble, puis tient. Poum. Le tunnel marche. Oui. Vous l'avez fait à deux. La limace a avancé d'un doigt. Le fil d'argent brille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut passer dans le tunnel. Moi, maintenant ! Il se glisse trop vite sous le carton. Le carton mouillé colle à son dos. Oh. Il reste collé. Un rire revient dans la bouche d'Aniss. Chouchou ne rit pas. Attends. Chouchou lâche le bord. Le carton s'écrase, une fois. Ça tombe ! Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le carton, un instant. Il écoute l'herbe, près du fil. Sur le fil, un &lt;emphasis level="moderate"&gt;éclat de limace&lt;/emphasis&gt; luit. Il est là. On tient, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Ils tiennent les deux bords, à deux. Aniss pousse le ballon, plus lent. Le ballon sort de l'autre côté. Il fait poum dans l'herbe. Il est passé ! Poum. Tu restes un peu ? Oui, papa. Le carton est près du banc. On le laisse ? Oui, contre le bois. Une goutte tombe du banc. Elle fait un rond dans l'eau. Un rond, maman. Oui, dans l'eau.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range le ballon. Delphine essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. [pause]</t>
+          <t>Aniss veut passer dans le tunnel. Moi, maintenant ! Il se glisse trop vite sous le carton. Le carton mouillé colle à son dos. Oh. Il reste collé. Un rire revient dans la bouche d'Aniss. Chouchou ne rit pas. Attends. Chouchou lâche le bord. Le carton s'écrase, une fois. Ça tombe ! Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le carton, un instant. Il écoute l'herbe, près du fil. Sur le fil, un &lt;emphasis&gt;éclat de limace&lt;/emphasis&gt; luit. Il est là. On tient, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Ils tiennent les deux bords, à deux. Aniss pousse le ballon, plus lent. Le ballon sort de l'autre côté. Il fait poum dans l'herbe. Il est passé ! Poum. Tu restes un peu ? Oui, papa. Le carton est près du banc. On le laisse ? Oui, contre le bois. Une goutte tombe du banc. Elle fait un rond dans l'eau. Un rond, maman. Oui, dans l'eau. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1821,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1829,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1855,30 +1918,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de limace</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,29 +1964,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sous_le_carton; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le ballon sort de l'autre côté.
+          <t>narrateur|Aniss veut passer dans le tunnel.
+enfant-m|Moi, maintenant !
+narrateur|Il se glisse trop vite sous le carton.
+narrateur|Le carton mouillé colle à son dos.
+enfant-m|Oh.
+enfant-f|Il reste collé.
+narrateur|Un rire revient dans la bouche d'Aniss.
+narrateur|Chouchou ne rit pas.
+enfant-f|Attends.
+narrateur|Chouchou lâche le bord.
+narrateur|Le carton s'écrase, une fois.
+enfant-m|Ça tombe !
+narrateur|Aniss avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Aniss refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le carton, un instant.
+narrateur|Il écoute l'herbe, près du fil.
+narrateur|Sur le fil, un éclat de limace luit.
+enfant-m|Il est là.
+enfant-m|On tient, si tu veux ?
+enfant-f|Plus tard.
+enfant-m|D'accord.
+narrateur|Chouchou s'approche, sans se presser.
+narrateur|Ils tiennent les deux bords, à deux.
+narrateur|Aniss pousse le ballon, plus lent.
+narrateur|Le ballon sort de l'autre côté.
 narrateur|Il fait poum dans l'herbe.
 enfant-m|Il est passé !
-copain|Poum.
-papa|Bravo.
-papa|Vous avez tenu le carton.
+enfant-f|Poum.
+papa|Tu restes un peu ?
+enfant-m|Oui, papa.
+maman|Le carton est près du banc.
+enfant-m|On le laisse ?
+papa|Oui, contre le bois.
 narrateur|Une goutte tombe du banc.
 narrateur|Elle fait un rond dans l'eau.
-papa|On le refait ?
-enfant-m|Encore.
-narrateur|Chouchou redresse le bord.
-narrateur|Aniss attend de l'autre côté.
-narrateur|Le ballon traverse encore.
-narrateur|Le carton tremble, puis tient.
-narrateur|Poum.
-enfant-m|Le tunnel marche.
-papa|Oui.
-papa|Vous l'avez fait à deux.
-narrateur|La limace a avancé d'un doigt.
-narrateur|Le fil d'argent brille encore.</t>
+enfant-m|Un rond, maman.
+maman|Oui, dans l'eau.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>ballon,herbe</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2042,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le carton repose contre le banc. Le ballon jaune attend dans l'herbe. Il a traversé le tunnel. Oui. Vous avez joué ensemble. La terre sent encore le champignon.</t>
+          <t>Le carton repose contre le banc. Le ballon jaune attend dans l'herbe. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, dans l'herbe. On est bien, ici. Aniss glisse le doigt sur le fil, sans se presser. On le voit, maman. Tu le vois sur le fil ? Oui, l'éclat. La limace a bougé, Aniss. Oui, d'un doigt. Elle est partie un peu. L'odeur de champignon reste sur le chemin. Il est là, maman. Oui, sur le fil. Un éclat de limace tient sur le fil.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le carton repose contre le banc. Le ballon jaune attend dans l'herbe. Il a traversé le tunnel. Oui. Vous avez joué ensemble. La terre sent encore le champignon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le carton repose contre le banc. Le ballon jaune attend dans l'herbe. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, dans l'herbe. On est bien, ici. Aniss glisse le doigt sur le fil, sans se presser. On le voit, maman. Tu le vois sur le fil ? Oui, l'éclat. La limace a bougé, Aniss. Oui, d'un doigt. Elle est partie un peu. L'odeur de champignon reste sur le chemin. Il est là, maman. Oui, sur le fil. Un &lt;emphasis level="moderate"&gt;éclat de limace&lt;/emphasis&gt; tient sur le fil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le carton repose contre le banc. Le ballon jaune attend dans l'herbe. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, dans l'herbe. On est bien, ici. Aniss glisse le doigt sur le fil, sans se presser. On le voit, maman. Tu le vois sur le fil ? Oui, l'éclat. La limace a bougé, Aniss. Oui, d'un doigt. Elle est partie un peu. L'odeur de champignon reste sur le chemin. Il est là, maman. Oui, sur le fil. Un &lt;emphasis&gt;éclat de limace&lt;/emphasis&gt; tient sur le fil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,18 +2099,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2119,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2133,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de limace</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2156,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,29 +2169,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fil; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Le carton repose contre le banc.
 narrateur|Le ballon jaune attend dans l'herbe.
-enfant-m|Il a traversé le tunnel.
-papa|Oui.
-papa|Vous avez joué ensemble.
-narrateur|La terre sent encore le champignon.</t>
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, dans l'herbe.
+maman|On est bien, ici.
+narrateur|Aniss glisse le doigt sur le fil, sans se presser.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le fil ?
+enfant-m|Oui, l'éclat.
+papa|La limace a bougé, Aniss.
+enfant-m|Oui, d'un doigt.
+enfant-f|Elle est partie un peu.
+narrateur|L'odeur de champignon reste sur le chemin.
+enfant-m|Il est là, maman.
+maman|Oui, sur le fil.
+narrateur|Un éclat de limace tient sur le fil.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>terre,limace</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2317,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>